<commit_message>
Adding Fred to code
</commit_message>
<xml_diff>
--- a/trades_taken.xlsx
+++ b/trades_taken.xlsx
@@ -548,7 +548,7 @@
         <v>5.749174382292647</v>
       </c>
       <c r="F2" t="n">
-        <v>1.141826279098585</v>
+        <v>1.141947091075164</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -591,7 +591,7 @@
         <v>5.773188699286039</v>
       </c>
       <c r="F3" t="n">
-        <v>1.134682625773983</v>
+        <v>1.134803942382518</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -644,7 +644,7 @@
         <v>5.78387729560523</v>
       </c>
       <c r="F4" t="n">
-        <v>1.105323031907443</v>
+        <v>1.105444573123957</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
@@ -697,7 +697,7 @@
         <v>5.793449133348831</v>
       </c>
       <c r="F5" t="n">
-        <v>1.097541426021955</v>
+        <v>1.097663168379113</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -750,7 +750,7 @@
         <v>5.803412368221555</v>
       </c>
       <c r="F6" t="n">
-        <v>1.090887357480231</v>
+        <v>1.091009309202772</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
@@ -803,7 +803,7 @@
         <v>5.815721008562775</v>
       </c>
       <c r="F7" t="n">
-        <v>1.086825520202334</v>
+        <v>1.08694773057613</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
@@ -856,7 +856,7 @@
         <v>5.815334021863411</v>
       </c>
       <c r="F8" t="n">
-        <v>1.072627019158087</v>
+        <v>1.072749221399825</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
@@ -909,7 +909,7 @@
         <v>5.806180843814804</v>
       </c>
       <c r="F9" t="n">
-        <v>1.100262632144622</v>
+        <v>1.100384642043344</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
@@ -962,7 +962,7 @@
         <v>5.797791852433679</v>
       </c>
       <c r="F10" t="n">
-        <v>1.101836173351318</v>
+        <v>1.101958006965488</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -1015,7 +1015,7 @@
         <v>5.773250764797821</v>
       </c>
       <c r="F11" t="n">
-        <v>1.074486443359815</v>
+        <v>1.07460776127258</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -1068,7 +1068,7 @@
         <v>5.792870686585944</v>
       </c>
       <c r="F12" t="n">
-        <v>1.089587472870435</v>
+        <v>1.089709203072231</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -1121,7 +1121,7 @@
         <v>5.799426812342785</v>
       </c>
       <c r="F13" t="n">
-        <v>1.093181360634961</v>
+        <v>1.093303228605845</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -1174,7 +1174,7 @@
         <v>5.791499330208546</v>
       </c>
       <c r="F14" t="n">
-        <v>1.114014641503429</v>
+        <v>1.114136342887822</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -1227,7 +1227,7 @@
         <v>5.807622181149471</v>
       </c>
       <c r="F15" t="n">
-        <v>1.096131873786599</v>
+        <v>1.09625391397329</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -1280,7 +1280,7 @@
         <v>5.811485489879658</v>
       </c>
       <c r="F16" t="n">
-        <v>1.104317652985041</v>
+        <v>1.104439774354512</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -1333,7 +1333,7 @@
         <v>5.815840058266167</v>
       </c>
       <c r="F17" t="n">
-        <v>1.11700838061204</v>
+        <v>1.117130593487522</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -1386,7 +1386,7 @@
         <v>5.822484503418294</v>
       </c>
       <c r="F18" t="n">
-        <v>1.117438125333774</v>
+        <v>1.11756047783427</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -1439,7 +1439,7 @@
         <v>5.821745073183263</v>
       </c>
       <c r="F19" t="n">
-        <v>1.110769841461688</v>
+        <v>1.110892178423948</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -1492,7 +1492,7 @@
         <v>5.838439218027872</v>
       </c>
       <c r="F20" t="n">
-        <v>1.069589211322751</v>
+        <v>1.069711899092362</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -1545,16 +1545,16 @@
         <v>5.826791450769824</v>
       </c>
       <c r="F21" t="n">
-        <v>1.049070440827043</v>
+        <v>1.049192883832851</v>
       </c>
       <c r="G21" t="n">
-        <v>1.098370375491807</v>
+        <v>1.098492297099277</v>
       </c>
       <c r="H21" t="n">
-        <v>0.02201289725452328</v>
+        <v>0.02201266124285643</v>
       </c>
       <c r="I21" t="n">
-        <v>-2.239593184610612</v>
+        <v>-2.239593510413244</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
@@ -1604,16 +1604,16 @@
         <v>5.806961871948709</v>
       </c>
       <c r="F22" t="n">
-        <v>1.028477897619893</v>
+        <v>1.02859992393098</v>
       </c>
       <c r="G22" t="n">
-        <v>1.092702956417872</v>
+        <v>1.092824938742068</v>
       </c>
       <c r="H22" t="n">
-        <v>0.02466719043036316</v>
+        <v>0.02466708176955401</v>
       </c>
       <c r="I22" t="n">
-        <v>-2.603663314607727</v>
+        <v>-2.603673000766515</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
@@ -1663,16 +1663,16 @@
         <v>5.801572597986273</v>
       </c>
       <c r="F23" t="n">
-        <v>1.018961128262691</v>
+        <v>1.019083041324676</v>
       </c>
       <c r="G23" t="n">
-        <v>1.086916881542308</v>
+        <v>1.087038893689176</v>
       </c>
       <c r="H23" t="n">
-        <v>0.02768899336895551</v>
+        <v>0.0276889659559465</v>
       </c>
       <c r="I23" t="n">
-        <v>-2.454251491706717</v>
+        <v>-2.454257499995431</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
@@ -1722,16 +1722,16 @@
         <v>5.775917931798511</v>
       </c>
       <c r="F24" t="n">
-        <v>1.112982141440127</v>
+        <v>1.113103515400194</v>
       </c>
       <c r="G24" t="n">
-        <v>1.087299837018942</v>
+        <v>1.087421840802988</v>
       </c>
       <c r="H24" t="n">
-        <v>0.02800808626306863</v>
+        <v>0.02800804431260939</v>
       </c>
       <c r="I24" t="n">
-        <v>0.9169603442363619</v>
+        <v>0.9169392304068992</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1781,16 +1781,16 @@
         <v>5.780429907926294</v>
       </c>
       <c r="F25" t="n">
-        <v>1.134437707914076</v>
+        <v>1.13455917668789</v>
       </c>
       <c r="G25" t="n">
-        <v>1.089144651113548</v>
+        <v>1.089266641218427</v>
       </c>
       <c r="H25" t="n">
-        <v>0.02987132666042008</v>
+        <v>0.02987124849863178</v>
       </c>
       <c r="I25" t="n">
-        <v>1.51627201949963</v>
+        <v>1.516258534407675</v>
       </c>
       <c r="J25" t="n">
         <v>-1</v>
@@ -1840,16 +1840,16 @@
         <v>5.762572732764129</v>
       </c>
       <c r="F26" t="n">
-        <v>1.139215016486785</v>
+        <v>1.139336110013565</v>
       </c>
       <c r="G26" t="n">
-        <v>1.091561034063875</v>
+        <v>1.091682981258966</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0319051664719824</v>
+        <v>0.03190502276937025</v>
       </c>
       <c r="I26" t="n">
-        <v>1.493613345185255</v>
+        <v>1.493593315982446</v>
       </c>
       <c r="J26" t="n">
         <v>-1</v>
@@ -1899,16 +1899,16 @@
         <v>5.738363354184461</v>
       </c>
       <c r="F27" t="n">
-        <v>1.164412077401906</v>
+        <v>1.164532662197749</v>
       </c>
       <c r="G27" t="n">
-        <v>1.095440361923854</v>
+        <v>1.095562227840047</v>
       </c>
       <c r="H27" t="n">
-        <v>0.0357805585519463</v>
+        <v>0.03578029552809846</v>
       </c>
       <c r="I27" t="n">
-        <v>1.927631045164332</v>
+        <v>1.927609410144153</v>
       </c>
       <c r="J27" t="n">
         <v>-1</v>
@@ -1958,16 +1958,16 @@
         <v>5.732040520720335</v>
       </c>
       <c r="F28" t="n">
-        <v>1.152409951745634</v>
+        <v>1.152530403674744</v>
       </c>
       <c r="G28" t="n">
-        <v>1.099429508553232</v>
+        <v>1.099551286953793</v>
       </c>
       <c r="H28" t="n">
-        <v>0.0375089735054342</v>
+        <v>0.03750863013418261</v>
       </c>
       <c r="I28" t="n">
-        <v>1.412473822690101</v>
+        <v>1.412451388691732</v>
       </c>
       <c r="J28" t="n">
         <v>-1</v>
@@ -2017,16 +2017,16 @@
         <v>5.721368826915722</v>
       </c>
       <c r="F29" t="n">
-        <v>1.137660216715829</v>
+        <v>1.137780444392145</v>
       </c>
       <c r="G29" t="n">
-        <v>1.101299387781792</v>
+        <v>1.101421077071233</v>
       </c>
       <c r="H29" t="n">
-        <v>0.03847248008936358</v>
+        <v>0.0384720685093613</v>
       </c>
       <c r="I29" t="n">
-        <v>0.9451126844325674</v>
+        <v>0.9450848038509821</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -2076,16 +2076,16 @@
         <v>5.70919231456057</v>
       </c>
       <c r="F30" t="n">
-        <v>1.15806762630886</v>
+        <v>1.158187598110431</v>
       </c>
       <c r="G30" t="n">
-        <v>1.104110960429669</v>
+        <v>1.10423255662848</v>
       </c>
       <c r="H30" t="n">
-        <v>0.04051429163818596</v>
+        <v>0.04051378084160917</v>
       </c>
       <c r="I30" t="n">
-        <v>1.33179339184929</v>
+        <v>1.331770088131027</v>
       </c>
       <c r="J30" t="n">
         <v>-1</v>
@@ -2135,16 +2135,16 @@
         <v>5.713520469255783</v>
       </c>
       <c r="F31" t="n">
-        <v>1.171130879586729</v>
+        <v>1.171250942339261</v>
       </c>
       <c r="G31" t="n">
-        <v>1.108943182241015</v>
+        <v>1.109064715681815</v>
       </c>
       <c r="H31" t="n">
-        <v>0.04250931719013069</v>
+        <v>0.04250870042499809</v>
       </c>
       <c r="I31" t="n">
-        <v>1.462919224685941</v>
+        <v>1.462905853053935</v>
       </c>
       <c r="J31" t="n">
         <v>-1</v>
@@ -2194,16 +2194,16 @@
         <v>5.711936800350696</v>
       </c>
       <c r="F32" t="n">
-        <v>1.171831704095611</v>
+        <v>1.171951733569247</v>
       </c>
       <c r="G32" t="n">
-        <v>1.113055393802273</v>
+        <v>1.113176842206665</v>
       </c>
       <c r="H32" t="n">
-        <v>0.04447111181121043</v>
+        <v>0.04447042310042733</v>
       </c>
       <c r="I32" t="n">
-        <v>1.321673956406944</v>
+        <v>1.321662517800895</v>
       </c>
       <c r="J32" t="n">
         <v>-1</v>
@@ -2253,16 +2253,16 @@
         <v>5.75120839641801</v>
       </c>
       <c r="F33" t="n">
-        <v>1.154064544717499</v>
+        <v>1.154185399436435</v>
       </c>
       <c r="G33" t="n">
-        <v>1.1160995530064</v>
+        <v>1.116220950748195</v>
       </c>
       <c r="H33" t="n">
-        <v>0.04511817878931619</v>
+        <v>0.04511748488006197</v>
       </c>
       <c r="I33" t="n">
-        <v>0.841456652946471</v>
+        <v>0.8414575588413939</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -2312,16 +2312,16 @@
         <v>5.740066355466205</v>
       </c>
       <c r="F34" t="n">
-        <v>1.171062320619905</v>
+        <v>1.171182941202269</v>
       </c>
       <c r="G34" t="n">
-        <v>1.118951936962224</v>
+        <v>1.119073280663917</v>
       </c>
       <c r="H34" t="n">
-        <v>0.04675309625049977</v>
+        <v>0.04675238270422814</v>
       </c>
       <c r="I34" t="n">
-        <v>1.114586793962845</v>
+        <v>1.11458833805361</v>
       </c>
       <c r="J34" t="n">
         <v>-1</v>
@@ -2371,16 +2371,16 @@
         <v>5.738170534486693</v>
       </c>
       <c r="F35" t="n">
-        <v>1.179174696136368</v>
+        <v>1.179295276880336</v>
       </c>
       <c r="G35" t="n">
-        <v>1.123104078079713</v>
+        <v>1.123225348809269</v>
       </c>
       <c r="H35" t="n">
-        <v>0.04828228840190949</v>
+        <v>0.04828157129980546</v>
       </c>
       <c r="I35" t="n">
-        <v>1.161308212856741</v>
+        <v>1.161311170320025</v>
       </c>
       <c r="J35" t="n">
         <v>-1</v>
@@ -2430,16 +2430,16 @@
         <v>5.744582886912311</v>
       </c>
       <c r="F36" t="n">
-        <v>1.188568094453422</v>
+        <v>1.188688809945255</v>
       </c>
       <c r="G36" t="n">
-        <v>1.127316600153132</v>
+        <v>1.127437800588806</v>
       </c>
       <c r="H36" t="n">
-        <v>0.05019441619225083</v>
+        <v>0.05019371126094478</v>
       </c>
       <c r="I36" t="n">
-        <v>1.220285022654504</v>
+        <v>1.220292499154316</v>
       </c>
       <c r="J36" t="n">
         <v>-1</v>
@@ -2489,16 +2489,16 @@
         <v>5.726783927032285</v>
       </c>
       <c r="F37" t="n">
-        <v>1.145122201880307</v>
+        <v>1.145242543348432</v>
       </c>
       <c r="G37" t="n">
-        <v>1.128722291216545</v>
+        <v>1.128843398081852</v>
       </c>
       <c r="H37" t="n">
-        <v>0.0502841241222951</v>
+        <v>0.0502834181170008</v>
       </c>
       <c r="I37" t="n">
-        <v>0.3261449006027446</v>
+        <v>0.3261342581847064</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -2548,16 +2548,16 @@
         <v>5.740932893433766</v>
       </c>
       <c r="F38" t="n">
-        <v>1.092519733490692</v>
+        <v>1.092640372282307</v>
       </c>
       <c r="G38" t="n">
-        <v>1.127476371624391</v>
+        <v>1.127597392804254</v>
       </c>
       <c r="H38" t="n">
-        <v>0.05088356994148131</v>
+        <v>0.05088290211111998</v>
       </c>
       <c r="I38" t="n">
-        <v>-0.6869926417093202</v>
+        <v>-0.6870091734470395</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -2607,16 +2607,16 @@
         <v>5.723982150556365</v>
       </c>
       <c r="F39" t="n">
-        <v>1.133994639076319</v>
+        <v>1.134114921668485</v>
       </c>
       <c r="G39" t="n">
-        <v>1.128637611505122</v>
+        <v>1.12875852996648</v>
       </c>
       <c r="H39" t="n">
-        <v>0.05074706432218951</v>
+        <v>0.05074641497452159</v>
       </c>
       <c r="I39" t="n">
-        <v>0.105563299921859</v>
+        <v>0.1055521203752783</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2666,16 +2666,16 @@
         <v>5.714344279418622</v>
       </c>
       <c r="F40" t="n">
-        <v>1.127443955042871</v>
+        <v>1.12756403510678</v>
       </c>
       <c r="G40" t="n">
-        <v>1.131530348691128</v>
+        <v>1.131651136767202</v>
       </c>
       <c r="H40" t="n">
-        <v>0.04881618524315948</v>
+        <v>0.04881563206320536</v>
       </c>
       <c r="I40" t="n">
-        <v>-0.08370981116001842</v>
+        <v>-0.08372526356166977</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2725,16 +2725,16 @@
         <v>5.712861012783621</v>
       </c>
       <c r="F41" t="n">
-        <v>1.144969116212413</v>
+        <v>1.14508916510726</v>
       </c>
       <c r="G41" t="n">
-        <v>1.136325282460397</v>
+        <v>1.136445950830922</v>
       </c>
       <c r="H41" t="n">
-        <v>0.04483802143781376</v>
+        <v>0.04483758117768515</v>
       </c>
       <c r="I41" t="n">
-        <v>0.1927791074368443</v>
+        <v>0.1927671843422123</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2784,16 +2784,16 @@
         <v>5.705410786907837</v>
       </c>
       <c r="F42" t="n">
-        <v>1.151905981487951</v>
+        <v>1.152025873825273</v>
       </c>
       <c r="G42" t="n">
-        <v>1.1424966866538</v>
+        <v>1.142617248325636</v>
       </c>
       <c r="H42" t="n">
-        <v>0.03702665493197799</v>
+        <v>0.03702633149706917</v>
       </c>
       <c r="I42" t="n">
-        <v>0.2541221952519609</v>
+        <v>0.2541063378201784</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2843,16 +2843,16 @@
         <v>5.697536098237152</v>
       </c>
       <c r="F43" t="n">
-        <v>1.126936811753264</v>
+        <v>1.127056538613487</v>
       </c>
       <c r="G43" t="n">
-        <v>1.147895470828328</v>
+        <v>1.148015923190077</v>
       </c>
       <c r="H43" t="n">
-        <v>0.02344829523849202</v>
+        <v>0.02344821487991332</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.8938244278270175</v>
+        <v>-0.8938584316090068</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2902,16 +2902,16 @@
         <v>5.724163671495992</v>
       </c>
       <c r="F44" t="n">
-        <v>1.134796653971521</v>
+        <v>1.134916940378131</v>
       </c>
       <c r="G44" t="n">
-        <v>1.148986196454898</v>
+        <v>1.149106594438974</v>
       </c>
       <c r="H44" t="n">
-        <v>0.02221364354159552</v>
+        <v>0.02221364291268626</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.6387760052423042</v>
+        <v>-0.6387810462524249</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
@@ -2961,16 +2961,16 @@
         <v>5.726380928450948</v>
       </c>
       <c r="F45" t="n">
-        <v>1.144759585041945</v>
+        <v>1.14487991804154</v>
       </c>
       <c r="G45" t="n">
-        <v>1.149502290311291</v>
+        <v>1.149622631506656</v>
       </c>
       <c r="H45" t="n">
-        <v>0.02197648491637061</v>
+        <v>0.02197652364951244</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.2158081825821639</v>
+        <v>-0.2158081751579287</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -3020,16 +3020,16 @@
         <v>5.731772886030789</v>
       </c>
       <c r="F46" t="n">
-        <v>1.147774604564161</v>
+        <v>1.147895050869251</v>
       </c>
       <c r="G46" t="n">
-        <v>1.14993026971516</v>
+        <v>1.150050578549441</v>
       </c>
       <c r="H46" t="n">
-        <v>0.02184857632867353</v>
+        <v>0.02184863416137732</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.09866387258238934</v>
+        <v>-0.0986573194584439</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
@@ -3079,16 +3079,16 @@
         <v>5.714949142745352</v>
       </c>
       <c r="F47" t="n">
-        <v>1.144084193628695</v>
+        <v>1.144204286403078</v>
       </c>
       <c r="G47" t="n">
-        <v>1.1489138755265</v>
+        <v>1.149034159759707</v>
       </c>
       <c r="H47" t="n">
-        <v>0.02161095990586548</v>
+        <v>0.02161101049974041</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.2234829882079531</v>
+        <v>-0.2234913243268649</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -3138,16 +3138,16 @@
         <v>5.710756593323133</v>
       </c>
       <c r="F48" t="n">
-        <v>1.131160174610352</v>
+        <v>1.131280179283359</v>
       </c>
       <c r="G48" t="n">
-        <v>1.147851386669736</v>
+        <v>1.147971648540138</v>
       </c>
       <c r="H48" t="n">
-        <v>0.02194974147897231</v>
+        <v>0.02194980064767979</v>
       </c>
       <c r="I48" t="n">
-        <v>-0.7604286399169319</v>
+        <v>-0.7604383076045458</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -3197,16 +3197,16 @@
         <v>5.721549023996647</v>
       </c>
       <c r="F49" t="n">
-        <v>1.139826493463808</v>
+        <v>1.139946724926748</v>
       </c>
       <c r="G49" t="n">
-        <v>1.147959700507135</v>
+        <v>1.148079962566868</v>
       </c>
       <c r="H49" t="n">
-        <v>0.02190209818964759</v>
+        <v>0.02190215723505423</v>
       </c>
       <c r="I49" t="n">
-        <v>-0.3713437394400494</v>
+        <v>-0.3713441353211905</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -3256,16 +3256,16 @@
         <v>5.738938545760967</v>
       </c>
       <c r="F50" t="n">
-        <v>1.120391751973521</v>
+        <v>1.120512348856322</v>
       </c>
       <c r="G50" t="n">
-        <v>1.146075906790368</v>
+        <v>1.146196200104163</v>
       </c>
       <c r="H50" t="n">
-        <v>0.02259620862942144</v>
+        <v>0.02259625393793602</v>
       </c>
       <c r="I50" t="n">
-        <v>-1.1366577127193</v>
+        <v>-1.136641999084675</v>
       </c>
       <c r="J50" t="n">
         <v>1</v>
@@ -3315,16 +3315,16 @@
         <v>5.728495630575953</v>
       </c>
       <c r="F51" t="n">
-        <v>1.119374361197232</v>
+        <v>1.119494738634745</v>
       </c>
       <c r="G51" t="n">
-        <v>1.143488080870893</v>
+        <v>1.143608389918937</v>
       </c>
       <c r="H51" t="n">
-        <v>0.02253940206033145</v>
+        <v>0.02253945762851689</v>
       </c>
       <c r="I51" t="n">
-        <v>-1.069847354828479</v>
+        <v>-1.069841683044033</v>
       </c>
       <c r="J51" t="n">
         <v>1</v>
@@ -3374,16 +3374,16 @@
         <v>5.726673971164641</v>
       </c>
       <c r="F52" t="n">
-        <v>1.110418153869186</v>
+        <v>1.11053849302672</v>
       </c>
       <c r="G52" t="n">
-        <v>1.140417403359572</v>
+        <v>1.140537727891811</v>
       </c>
       <c r="H52" t="n">
-        <v>0.02265780468105381</v>
+        <v>0.02265787826162289</v>
       </c>
       <c r="I52" t="n">
-        <v>-1.324013950719179</v>
+        <v>-1.324009005552044</v>
       </c>
       <c r="J52" t="n">
         <v>1</v>
@@ -3433,16 +3433,16 @@
         <v>5.706513118053733</v>
       </c>
       <c r="F53" t="n">
-        <v>1.091389717338871</v>
+        <v>1.091509632840355</v>
       </c>
       <c r="G53" t="n">
-        <v>1.13728366199064</v>
+        <v>1.137403939562007</v>
       </c>
       <c r="H53" t="n">
-        <v>0.0248947352035948</v>
+        <v>0.02489482304977883</v>
       </c>
       <c r="I53" t="n">
-        <v>-1.843520096777005</v>
+        <v>-1.843528135543815</v>
       </c>
       <c r="J53" t="n">
         <v>1</v>
@@ -3492,16 +3492,16 @@
         <v>5.710028592673332</v>
       </c>
       <c r="F54" t="n">
-        <v>1.105769686989136</v>
+        <v>1.105889676364086</v>
       </c>
       <c r="G54" t="n">
-        <v>1.134019030309102</v>
+        <v>1.134139276320097</v>
       </c>
       <c r="H54" t="n">
-        <v>0.02451013261744044</v>
+        <v>0.02451021203965659</v>
       </c>
       <c r="I54" t="n">
-        <v>-1.152557750742826</v>
+        <v>-1.152564486602757</v>
       </c>
       <c r="J54" t="n">
         <v>1</v>
@@ -3551,16 +3551,16 @@
         <v>5.670799921537744</v>
       </c>
       <c r="F55" t="n">
-        <v>1.13116442567198</v>
+        <v>1.131283590703644</v>
       </c>
       <c r="G55" t="n">
-        <v>1.131618516785882</v>
+        <v>1.131738692011263</v>
       </c>
       <c r="H55" t="n">
-        <v>0.02208601692115957</v>
+        <v>0.02208606829704957</v>
       </c>
       <c r="I55" t="n">
-        <v>-0.02056011799333949</v>
+        <v>-0.02060580912355634</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
@@ -3610,16 +3610,16 @@
         <v>5.672485518208908</v>
       </c>
       <c r="F56" t="n">
-        <v>1.149633810870154</v>
+        <v>1.149753011322602</v>
       </c>
       <c r="G56" t="n">
-        <v>1.129671802606719</v>
+        <v>1.12979190208013</v>
       </c>
       <c r="H56" t="n">
-        <v>0.01817104873131073</v>
+        <v>0.01817096265221098</v>
       </c>
       <c r="I56" t="n">
-        <v>1.098561153987668</v>
+        <v>1.098516882375687</v>
       </c>
       <c r="J56" t="n">
         <v>-1</v>
@@ -3669,16 +3669,16 @@
         <v>5.63747285479881</v>
       </c>
       <c r="F57" t="n">
-        <v>1.132007756532976</v>
+        <v>1.132126221236463</v>
       </c>
       <c r="G57" t="n">
-        <v>1.129016080339353</v>
+        <v>1.129136085974532</v>
       </c>
       <c r="H57" t="n">
-        <v>0.01781734169597524</v>
+        <v>0.01781722795127691</v>
       </c>
       <c r="I57" t="n">
-        <v>0.16790811135978</v>
+        <v>0.1678226977904937</v>
       </c>
       <c r="J57" t="n">
         <v>0</v>
@@ -3728,16 +3728,16 @@
         <v>5.613771107697508</v>
       </c>
       <c r="F58" t="n">
-        <v>1.126903223657087</v>
+        <v>1.127021190296901</v>
       </c>
       <c r="G58" t="n">
-        <v>1.130735254847672</v>
+        <v>1.130855126875262</v>
       </c>
       <c r="H58" t="n">
-        <v>0.01563576407735688</v>
+        <v>0.01563574221715024</v>
       </c>
       <c r="I58" t="n">
-        <v>-0.2450811595535944</v>
+        <v>-0.2452033632375522</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
@@ -3787,16 +3787,16 @@
         <v>5.610704481843535</v>
       </c>
       <c r="F59" t="n">
-        <v>1.11495702046316</v>
+        <v>1.115074922661524</v>
       </c>
       <c r="G59" t="n">
-        <v>1.129783373917014</v>
+        <v>1.129903126924913</v>
       </c>
       <c r="H59" t="n">
-        <v>0.01600209327752923</v>
+        <v>0.0160021622942953</v>
       </c>
       <c r="I59" t="n">
-        <v>-0.926525873628945</v>
+        <v>-0.9266375375205114</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
@@ -3846,16 +3846,16 @@
         <v>5.66083438890224</v>
       </c>
       <c r="F60" t="n">
-        <v>1.133676236566434</v>
+        <v>1.13379519218443</v>
       </c>
       <c r="G60" t="n">
-        <v>1.130094987993192</v>
+        <v>1.130214684778796</v>
       </c>
       <c r="H60" t="n">
-        <v>0.01601481588418293</v>
+        <v>0.01601487831146685</v>
       </c>
       <c r="I60" t="n">
-        <v>0.223620964433258</v>
+        <v>0.2235738128007271</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
@@ -3905,16 +3905,16 @@
         <v>5.694447350642657</v>
       </c>
       <c r="F61" t="n">
-        <v>1.117478634064746</v>
+        <v>1.117598296018657</v>
       </c>
       <c r="G61" t="n">
-        <v>1.128720463885809</v>
+        <v>1.128840141324366</v>
       </c>
       <c r="H61" t="n">
-        <v>0.01584988559482496</v>
+        <v>0.01584993097350644</v>
       </c>
       <c r="I61" t="n">
-        <v>-0.709268830604905</v>
+        <v>-0.709267776907046</v>
       </c>
       <c r="J61" t="n">
         <v>0</v>
@@ -3964,16 +3964,16 @@
         <v>5.688985012996693</v>
       </c>
       <c r="F62" t="n">
-        <v>1.130652043465206</v>
+        <v>1.130771590634669</v>
       </c>
       <c r="G62" t="n">
-        <v>1.127657766984672</v>
+        <v>1.127777427164836</v>
       </c>
       <c r="H62" t="n">
-        <v>0.01489742979091636</v>
+        <v>0.0148974582829823</v>
       </c>
       <c r="I62" t="n">
-        <v>0.2009928237661461</v>
+        <v>0.2009848534534332</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -4023,16 +4023,16 @@
         <v>5.703151986226595</v>
       </c>
       <c r="F63" t="n">
-        <v>1.121983516373925</v>
+        <v>1.122103361245271</v>
       </c>
       <c r="G63" t="n">
-        <v>1.127410102215705</v>
+        <v>1.127529768296425</v>
       </c>
       <c r="H63" t="n">
-        <v>0.01495112292899852</v>
+        <v>0.01495114790175834</v>
       </c>
       <c r="I63" t="n">
-        <v>-0.3629550681611027</v>
+        <v>-0.362942503599702</v>
       </c>
       <c r="J63" t="n">
         <v>0</v>
@@ -4082,16 +4082,16 @@
         <v>5.721221686860314</v>
       </c>
       <c r="F64" t="n">
-        <v>1.111716875117168</v>
+        <v>1.111837099701513</v>
       </c>
       <c r="G64" t="n">
-        <v>1.126256113272987</v>
+        <v>1.126375776262594</v>
       </c>
       <c r="H64" t="n">
-        <v>0.01523891811370703</v>
+        <v>0.01523889627168938</v>
       </c>
       <c r="I64" t="n">
-        <v>-0.9540859821761901</v>
+        <v>-0.9540504969569495</v>
       </c>
       <c r="J64" t="n">
         <v>0</v>
@@ -4141,16 +4141,16 @@
         <v>5.759313628223341</v>
       </c>
       <c r="F65" t="n">
-        <v>1.106723344363796</v>
+        <v>1.106844369404419</v>
       </c>
       <c r="G65" t="n">
-        <v>1.12435430123908</v>
+        <v>1.124473998830738</v>
       </c>
       <c r="H65" t="n">
-        <v>0.01518149963773092</v>
+        <v>0.01518134706401714</v>
       </c>
       <c r="I65" t="n">
-        <v>-1.161344880018659</v>
+        <v>-1.161269112153095</v>
       </c>
       <c r="J65" t="n">
         <v>1</v>
@@ -4200,16 +4200,16 @@
         <v>5.762993912430139</v>
       </c>
       <c r="F66" t="n">
-        <v>1.1141059190858</v>
+        <v>1.114227021463163</v>
       </c>
       <c r="G66" t="n">
-        <v>1.122670866965162</v>
+        <v>1.122790597360434</v>
       </c>
       <c r="H66" t="n">
-        <v>0.01428823661100067</v>
+        <v>0.01428796094483416</v>
       </c>
       <c r="I66" t="n">
-        <v>-0.5994405126779365</v>
+        <v>-0.5993560543967172</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
@@ -4259,16 +4259,16 @@
         <v>5.759061472992551</v>
       </c>
       <c r="F67" t="n">
-        <v>1.142243965822793</v>
+        <v>1.142364985564678</v>
       </c>
       <c r="G67" t="n">
-        <v>1.122578855574867</v>
+        <v>1.122698632318514</v>
       </c>
       <c r="H67" t="n">
-        <v>0.01414832465767295</v>
+        <v>0.01414811159993049</v>
       </c>
       <c r="I67" t="n">
-        <v>1.389925006934412</v>
+        <v>1.390033794069074</v>
       </c>
       <c r="J67" t="n">
         <v>-1</v>
@@ -4318,16 +4318,16 @@
         <v>5.771809262772875</v>
       </c>
       <c r="F68" t="n">
-        <v>1.136774965406905</v>
+        <v>1.136896253028241</v>
       </c>
       <c r="G68" t="n">
-        <v>1.122859595114694</v>
+        <v>1.122979436005757</v>
       </c>
       <c r="H68" t="n">
-        <v>0.01438134926315747</v>
+        <v>0.01438120968180669</v>
       </c>
       <c r="I68" t="n">
-        <v>0.967598382987626</v>
+        <v>0.9677083729673678</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -4377,16 +4377,16 @@
         <v>5.807275066409984</v>
       </c>
       <c r="F69" t="n">
-        <v>1.14887584285261</v>
+        <v>1.148997875745103</v>
       </c>
       <c r="G69" t="n">
-        <v>1.123312062584134</v>
+        <v>1.123431993546675</v>
       </c>
       <c r="H69" t="n">
-        <v>0.01506916666662325</v>
+        <v>0.01506920665133907</v>
       </c>
       <c r="I69" t="n">
-        <v>1.696429592559829</v>
+        <v>1.696564576354485</v>
       </c>
       <c r="J69" t="n">
         <v>-1</v>
@@ -4436,16 +4436,16 @@
         <v>5.819841839592116</v>
       </c>
       <c r="F70" t="n">
-        <v>1.151875219551731</v>
+        <v>1.151997516519829</v>
       </c>
       <c r="G70" t="n">
-        <v>1.124886235963045</v>
+        <v>1.125006251929851</v>
       </c>
       <c r="H70" t="n">
-        <v>0.01633897694062399</v>
+        <v>0.01633922916011205</v>
       </c>
       <c r="I70" t="n">
-        <v>1.65181600333756</v>
+        <v>1.651930107931327</v>
       </c>
       <c r="J70" t="n">
         <v>-1</v>
@@ -4495,16 +4495,16 @@
         <v>5.816573506443499</v>
       </c>
       <c r="F71" t="n">
-        <v>1.151581766950863</v>
+        <v>1.151703995238876</v>
       </c>
       <c r="G71" t="n">
-        <v>1.126496606250726</v>
+        <v>1.126616714760057</v>
       </c>
       <c r="H71" t="n">
-        <v>0.01732458846458469</v>
+        <v>0.01732500275663296</v>
       </c>
       <c r="I71" t="n">
-        <v>1.447951317944228</v>
+        <v>1.448039046874823</v>
       </c>
       <c r="J71" t="n">
         <v>-1</v>
@@ -4554,16 +4554,16 @@
         <v>5.833277526334015</v>
       </c>
       <c r="F72" t="n">
-        <v>1.156349392018983</v>
+        <v>1.156471971321859</v>
       </c>
       <c r="G72" t="n">
-        <v>1.128793168158216</v>
+        <v>1.128913388674814</v>
       </c>
       <c r="H72" t="n">
-        <v>0.01810768112550796</v>
+        <v>0.01810828771974418</v>
       </c>
       <c r="I72" t="n">
-        <v>1.521797499622897</v>
+        <v>1.52187678225351</v>
       </c>
       <c r="J72" t="n">
         <v>-1</v>
@@ -4613,16 +4613,16 @@
         <v>5.820731377074562</v>
       </c>
       <c r="F73" t="n">
-        <v>1.167155800802261</v>
+        <v>1.167278116462918</v>
       </c>
       <c r="G73" t="n">
-        <v>1.132581472331386</v>
+        <v>1.132701812855942</v>
       </c>
       <c r="H73" t="n">
-        <v>0.01779343858832908</v>
+        <v>0.0177942329967179</v>
       </c>
       <c r="I73" t="n">
-        <v>1.943094264733797</v>
+        <v>1.943118515608581</v>
       </c>
       <c r="J73" t="n">
         <v>-1</v>
@@ -4672,16 +4672,16 @@
         <v>5.805410967834648</v>
       </c>
       <c r="F74" t="n">
-        <v>1.167205688743451</v>
+        <v>1.167327682464157</v>
       </c>
       <c r="G74" t="n">
-        <v>1.135653272419102</v>
+        <v>1.135773713160946</v>
       </c>
       <c r="H74" t="n">
-        <v>0.01821908786853837</v>
+        <v>0.01821998408930763</v>
       </c>
       <c r="I74" t="n">
-        <v>1.731832929947911</v>
+        <v>1.731832977929323</v>
       </c>
       <c r="J74" t="n">
         <v>-1</v>
@@ -4731,16 +4731,16 @@
         <v>5.826346543406457</v>
       </c>
       <c r="F75" t="n">
-        <v>1.165337032295263</v>
+        <v>1.165459465951879</v>
       </c>
       <c r="G75" t="n">
-        <v>1.137361902750265</v>
+        <v>1.137482506923358</v>
       </c>
       <c r="H75" t="n">
-        <v>0.01934364521730167</v>
+        <v>0.019344619516754</v>
       </c>
       <c r="I75" t="n">
-        <v>1.44621808509887</v>
+        <v>1.446239818999344</v>
       </c>
       <c r="J75" t="n">
         <v>-1</v>
@@ -4790,16 +4790,16 @@
         <v>5.825078484064047</v>
       </c>
       <c r="F76" t="n">
-        <v>1.152014833917419</v>
+        <v>1.152137240927295</v>
       </c>
       <c r="G76" t="n">
-        <v>1.137480953902629</v>
+        <v>1.137601718403592</v>
       </c>
       <c r="H76" t="n">
-        <v>0.01943028129778861</v>
+        <v>0.0194313684320313</v>
       </c>
       <c r="I76" t="n">
-        <v>0.7480015236034899</v>
+        <v>0.7480442036054273</v>
       </c>
       <c r="J76" t="n">
         <v>0</v>
@@ -4849,16 +4849,16 @@
         <v>5.841206605238948</v>
       </c>
       <c r="F77" t="n">
-        <v>1.182862568276891</v>
+        <v>1.182985314199811</v>
       </c>
       <c r="G77" t="n">
-        <v>1.140023694489825</v>
+        <v>1.14014467305176</v>
       </c>
       <c r="H77" t="n">
-        <v>0.02185286351801664</v>
+        <v>0.02185399016318637</v>
       </c>
       <c r="I77" t="n">
-        <v>1.960332281018795</v>
+        <v>1.960312090751177</v>
       </c>
       <c r="J77" t="n">
         <v>-1</v>
@@ -4908,16 +4908,16 @@
         <v>5.858306968534851</v>
       </c>
       <c r="F78" t="n">
-        <v>1.209962394099189</v>
+        <v>1.210085499365652</v>
       </c>
       <c r="G78" t="n">
-        <v>1.14417665301193</v>
+        <v>1.144297888505197</v>
       </c>
       <c r="H78" t="n">
-        <v>0.026604054789146</v>
+        <v>0.02660515408000967</v>
       </c>
       <c r="I78" t="n">
-        <v>2.47277122260696</v>
+        <v>2.472739329477735</v>
       </c>
       <c r="J78" t="n">
         <v>-1</v>
@@ -4967,16 +4967,16 @@
         <v>5.85670725340159</v>
       </c>
       <c r="F79" t="n">
-        <v>1.195091755715976</v>
+        <v>1.195214827366352</v>
       </c>
       <c r="G79" t="n">
-        <v>1.148183389774571</v>
+        <v>1.148304883740439</v>
       </c>
       <c r="H79" t="n">
-        <v>0.02797105727884313</v>
+        <v>0.02797205651019888</v>
       </c>
       <c r="I79" t="n">
-        <v>1.677032279251234</v>
+        <v>1.677028773655226</v>
       </c>
       <c r="J79" t="n">
         <v>-1</v>
@@ -5026,16 +5026,16 @@
         <v>5.857164600990844</v>
       </c>
       <c r="F80" t="n">
-        <v>1.176206191718337</v>
+        <v>1.176329272979323</v>
       </c>
       <c r="G80" t="n">
-        <v>1.150309887532166</v>
+        <v>1.150431587780183</v>
       </c>
       <c r="H80" t="n">
-        <v>0.02842311970445721</v>
+        <v>0.02842410097128862</v>
       </c>
       <c r="I80" t="n">
-        <v>0.9110999937881666</v>
+        <v>0.9111171264589403</v>
       </c>
       <c r="J80" t="n">
         <v>0</v>
@@ -5085,16 +5085,16 @@
         <v>5.952126560232704</v>
       </c>
       <c r="F81" t="n">
-        <v>1.061295779403068</v>
+        <v>1.061420856175275</v>
       </c>
       <c r="G81" t="n">
-        <v>1.147500744799082</v>
+        <v>1.147622715788014</v>
       </c>
       <c r="H81" t="n">
-        <v>0.03405676030334023</v>
+        <v>0.03405703487114223</v>
       </c>
       <c r="I81" t="n">
-        <v>-2.531214496863318</v>
+        <v>-2.53110289662303</v>
       </c>
       <c r="J81" t="n">
         <v>1</v>
@@ -5144,16 +5144,16 @@
         <v>5.954436849899731</v>
       </c>
       <c r="F82" t="n">
-        <v>1.054024604611568</v>
+        <v>1.05414972993173</v>
       </c>
       <c r="G82" t="n">
-        <v>1.1436693728564</v>
+        <v>1.143791622752867</v>
       </c>
       <c r="H82" t="n">
-        <v>0.03986669719088096</v>
+        <v>0.03986651678390481</v>
       </c>
       <c r="I82" t="n">
-        <v>-2.248612866413649</v>
+        <v>-2.24855091572304</v>
       </c>
       <c r="J82" t="n">
         <v>1</v>
@@ -5203,16 +5203,16 @@
         <v>5.948090365497994</v>
       </c>
       <c r="F83" t="n">
-        <v>1.058689912217301</v>
+        <v>1.058814904173736</v>
       </c>
       <c r="G83" t="n">
-        <v>1.140504692648569</v>
+        <v>1.14062719989929</v>
       </c>
       <c r="H83" t="n">
-        <v>0.04397884999816178</v>
+        <v>0.04397836467034311</v>
       </c>
       <c r="I83" t="n">
-        <v>-1.860321050566064</v>
+        <v>-1.860285081967242</v>
       </c>
       <c r="J83" t="n">
         <v>1</v>
@@ -5262,16 +5262,16 @@
         <v>5.961515828160556</v>
       </c>
       <c r="F84" t="n">
-        <v>1.039114586461601</v>
+        <v>1.039239860537966</v>
       </c>
       <c r="G84" t="n">
-        <v>1.13687457821579</v>
+        <v>1.136997337941113</v>
       </c>
       <c r="H84" t="n">
-        <v>0.04917011623169936</v>
+        <v>0.04916933114470609</v>
       </c>
       <c r="I84" t="n">
-        <v>-1.988199321993156</v>
+        <v>-1.988179931011161</v>
       </c>
       <c r="J84" t="n">
         <v>1</v>
@@ -5321,16 +5321,16 @@
         <v>5.98595539627007</v>
       </c>
       <c r="F85" t="n">
-        <v>1.077788945347342</v>
+        <v>1.077914732991801</v>
       </c>
       <c r="G85" t="n">
-        <v>1.135427858264968</v>
+        <v>1.135550856120482</v>
       </c>
       <c r="H85" t="n">
-        <v>0.0505113126520777</v>
+        <v>0.05051031467459768</v>
       </c>
       <c r="I85" t="n">
-        <v>-1.141108989082174</v>
+        <v>-1.141076302929208</v>
       </c>
       <c r="J85" t="n">
         <v>1</v>
@@ -5380,16 +5380,16 @@
         <v>5.985829728516112</v>
       </c>
       <c r="F86" t="n">
-        <v>1.095382883438691</v>
+        <v>1.095508668442394</v>
       </c>
       <c r="G86" t="n">
-        <v>1.134491706482612</v>
+        <v>1.134614938469444</v>
       </c>
       <c r="H86" t="n">
-        <v>0.05109738314762458</v>
+        <v>0.05109624453940078</v>
       </c>
       <c r="I86" t="n">
-        <v>-0.7653781981541506</v>
+        <v>-0.7653452886717393</v>
       </c>
       <c r="J86" t="n">
         <v>0</v>
@@ -5439,16 +5439,16 @@
         <v>5.992865390419841</v>
       </c>
       <c r="F87" t="n">
-        <v>1.1077213039358</v>
+        <v>1.107847236785466</v>
       </c>
       <c r="G87" t="n">
-        <v>1.132765573388262</v>
+        <v>1.132889051030483</v>
       </c>
       <c r="H87" t="n">
-        <v>0.05140390879291727</v>
+        <v>0.05140272918670828</v>
       </c>
       <c r="I87" t="n">
-        <v>-0.4872055460481514</v>
+        <v>-0.487168962450576</v>
       </c>
       <c r="J87" t="n">
         <v>0</v>
@@ -5498,16 +5498,16 @@
         <v>5.962056385069926</v>
       </c>
       <c r="F88" t="n">
-        <v>1.149146533404532</v>
+        <v>1.149271818840051</v>
       </c>
       <c r="G88" t="n">
-        <v>1.133384151788144</v>
+        <v>1.133507829321074</v>
       </c>
       <c r="H88" t="n">
-        <v>0.05152898151657757</v>
+        <v>0.05152784146295274</v>
       </c>
       <c r="I88" t="n">
-        <v>0.305893521518902</v>
+        <v>0.3059314939538245</v>
       </c>
       <c r="J88" t="n">
         <v>0</v>
@@ -5557,16 +5557,16 @@
         <v>5.958731556573001</v>
       </c>
       <c r="F89" t="n">
-        <v>1.15759934330762</v>
+        <v>1.157724558875872</v>
       </c>
       <c r="G89" t="n">
-        <v>1.133820326810894</v>
+        <v>1.133944163477612</v>
       </c>
       <c r="H89" t="n">
-        <v>0.05170363970790831</v>
+        <v>0.05170256594109949</v>
       </c>
       <c r="I89" t="n">
-        <v>0.4599099141000788</v>
+        <v>0.4599461354655137</v>
       </c>
       <c r="J89" t="n">
         <v>0</v>
@@ -5616,16 +5616,16 @@
         <v>5.997396093626087</v>
       </c>
       <c r="F90" t="n">
-        <v>1.152713344230624</v>
+        <v>1.152839372287562</v>
       </c>
       <c r="G90" t="n">
-        <v>1.133862233044839</v>
+        <v>1.133986256265999</v>
       </c>
       <c r="H90" t="n">
-        <v>0.05171938079907197</v>
+        <v>0.0517183776238547</v>
       </c>
       <c r="I90" t="n">
-        <v>0.3644883386949449</v>
+        <v>0.3645341731073014</v>
       </c>
       <c r="J90" t="n">
         <v>0</v>
@@ -5675,16 +5675,16 @@
         <v>5.993538886487244</v>
       </c>
       <c r="F91" t="n">
-        <v>1.198403965306636</v>
+        <v>1.198529912309011</v>
       </c>
       <c r="G91" t="n">
-        <v>1.136203342962627</v>
+        <v>1.136327552119506</v>
       </c>
       <c r="H91" t="n">
-        <v>0.05358958562568128</v>
+        <v>0.05358876209393353</v>
       </c>
       <c r="I91" t="n">
-        <v>1.160684890875531</v>
+        <v>1.160735157130024</v>
       </c>
       <c r="J91" t="n">
         <v>-1</v>
@@ -5734,16 +5734,16 @@
         <v>5.982784867071093</v>
       </c>
       <c r="F92" t="n">
-        <v>1.160845344567659</v>
+        <v>1.160971065587266</v>
       </c>
       <c r="G92" t="n">
-        <v>1.136428140590061</v>
+        <v>1.136552506832776</v>
       </c>
       <c r="H92" t="n">
-        <v>0.05368788177202295</v>
+        <v>0.05368712776772819</v>
       </c>
       <c r="I92" t="n">
-        <v>0.4547991682980042</v>
+        <v>0.4548307903550858</v>
       </c>
       <c r="J92" t="n">
         <v>0</v>
@@ -5793,16 +5793,16 @@
         <v>5.983188051122531</v>
       </c>
       <c r="F93" t="n">
-        <v>1.14715474314571</v>
+        <v>1.147280472637744</v>
       </c>
       <c r="G93" t="n">
-        <v>1.135428087707234</v>
+        <v>1.135552624641517</v>
       </c>
       <c r="H93" t="n">
-        <v>0.05327004348207891</v>
+        <v>0.05326936363834962</v>
       </c>
       <c r="I93" t="n">
-        <v>0.2201360215225118</v>
+        <v>0.2201612182914076</v>
       </c>
       <c r="J93" t="n">
         <v>0</v>
@@ -5852,16 +5852,16 @@
         <v>5.959531545016149</v>
       </c>
       <c r="F94" t="n">
-        <v>1.156260033838677</v>
+        <v>1.156385266217722</v>
       </c>
       <c r="G94" t="n">
-        <v>1.134880804961995</v>
+        <v>1.135005503829196</v>
       </c>
       <c r="H94" t="n">
-        <v>0.05298183243886066</v>
+        <v>0.05298124533018352</v>
       </c>
       <c r="I94" t="n">
-        <v>0.4035199971868288</v>
+        <v>0.4035345385954198</v>
       </c>
       <c r="J94" t="n">
         <v>0</v>
@@ -5911,16 +5911,16 @@
         <v>5.962750867995942</v>
       </c>
       <c r="F95" t="n">
-        <v>1.166850909122108</v>
+        <v>1.16697620915135</v>
       </c>
       <c r="G95" t="n">
-        <v>1.134956498803337</v>
+        <v>1.135081340989169</v>
       </c>
       <c r="H95" t="n">
-        <v>0.0530286953046184</v>
+        <v>0.05302819604618215</v>
       </c>
       <c r="I95" t="n">
-        <v>0.6014556861253436</v>
+        <v>0.6014699827692328</v>
       </c>
       <c r="J95" t="n">
         <v>0</v>
@@ -5970,16 +5970,16 @@
         <v>5.959531545016149</v>
       </c>
       <c r="F96" t="n">
-        <v>1.151261364278356</v>
+        <v>1.1513865966574</v>
       </c>
       <c r="G96" t="n">
-        <v>1.134918825321384</v>
+        <v>1.135043808775674</v>
       </c>
       <c r="H96" t="n">
-        <v>0.05301620479376808</v>
+        <v>0.05301575307530886</v>
       </c>
       <c r="I96" t="n">
-        <v>0.3082555422543675</v>
+        <v>0.3082628640304559</v>
       </c>
       <c r="J96" t="n">
         <v>0</v>
@@ -6029,16 +6029,16 @@
         <v>5.94735954974672</v>
       </c>
       <c r="F97" t="n">
-        <v>1.140693202264512</v>
+        <v>1.140818178863733</v>
       </c>
       <c r="G97" t="n">
-        <v>1.132810357020765</v>
+        <v>1.13293545200887</v>
       </c>
       <c r="H97" t="n">
-        <v>0.0518344884237897</v>
+        <v>0.05183414006595252</v>
       </c>
       <c r="I97" t="n">
-        <v>0.1520772266390961</v>
+        <v>0.1520759646988046</v>
       </c>
       <c r="J97" t="n">
         <v>0</v>
@@ -6088,16 +6088,16 @@
         <v>5.962673683416126</v>
       </c>
       <c r="F98" t="n">
-        <v>1.127615292588263</v>
+        <v>1.127740590995563</v>
       </c>
       <c r="G98" t="n">
-        <v>1.128693001945219</v>
+        <v>1.128818206590366</v>
       </c>
       <c r="H98" t="n">
-        <v>0.04855001177608873</v>
+        <v>0.04854981491006437</v>
       </c>
       <c r="I98" t="n">
-        <v>-0.02219792163854965</v>
+        <v>-0.02219608039287325</v>
       </c>
       <c r="J98" t="n">
         <v>0</v>
@@ -6147,16 +6147,16 @@
         <v>5.962545055387006</v>
       </c>
       <c r="F99" t="n">
-        <v>1.117132593241973</v>
+        <v>1.117257888946309</v>
       </c>
       <c r="G99" t="n">
-        <v>1.124795043821519</v>
+        <v>1.124920359669364</v>
       </c>
       <c r="H99" t="n">
-        <v>0.04600110766521245</v>
+        <v>0.04600107064509103</v>
       </c>
       <c r="I99" t="n">
-        <v>-0.1665710016226581</v>
+        <v>-0.166571573565588</v>
       </c>
       <c r="J99" t="n">
         <v>0</v>
@@ -6206,16 +6206,16 @@
         <v>5.965882922901972</v>
       </c>
       <c r="F100" t="n">
-        <v>1.12248944685128</v>
+        <v>1.122614812696884</v>
       </c>
       <c r="G100" t="n">
-        <v>1.122109206578166</v>
+        <v>1.122234636655242</v>
       </c>
       <c r="H100" t="n">
-        <v>0.04438104825347484</v>
+        <v>0.04438115325839519</v>
       </c>
       <c r="I100" t="n">
-        <v>0.008567627130901973</v>
+        <v>0.008566159590953464</v>
       </c>
       <c r="J100" t="n">
         <v>0</v>
@@ -6265,16 +6265,16 @@
         <v>5.940468433706842</v>
       </c>
       <c r="F101" t="n">
-        <v>1.125944501473731</v>
+        <v>1.126069333264446</v>
       </c>
       <c r="G101" t="n">
-        <v>1.125341642681699</v>
+        <v>1.1254670605097</v>
       </c>
       <c r="H101" t="n">
-        <v>0.04200960738259412</v>
+        <v>0.04200968951430623</v>
       </c>
       <c r="I101" t="n">
-        <v>0.01435049812632295</v>
+        <v>0.01433652001976859</v>
       </c>
       <c r="J101" t="n">
         <v>0</v>
@@ -6324,16 +6324,16 @@
         <v>5.929975570597685</v>
       </c>
       <c r="F102" t="n">
-        <v>1.194138458809176</v>
+        <v>1.19426307010501</v>
       </c>
       <c r="G102" t="n">
-        <v>1.132347335391579</v>
+        <v>1.132472727518364</v>
       </c>
       <c r="H102" t="n">
-        <v>0.04116502253103407</v>
+        <v>0.04116501333812039</v>
       </c>
       <c r="I102" t="n">
-        <v>1.501058899482267</v>
+        <v>1.501040266381391</v>
       </c>
       <c r="J102" t="n">
         <v>-1</v>
@@ -6383,16 +6383,16 @@
         <v>5.890632658072621</v>
       </c>
       <c r="F103" t="n">
-        <v>1.215235149844114</v>
+        <v>1.215358934396017</v>
       </c>
       <c r="G103" t="n">
-        <v>1.14017459727292</v>
+        <v>1.140299929029478</v>
       </c>
       <c r="H103" t="n">
-        <v>0.04130520277187692</v>
+        <v>0.04130499830860931</v>
       </c>
       <c r="I103" t="n">
-        <v>1.817217869277702</v>
+        <v>1.817189406612167</v>
       </c>
       <c r="J103" t="n">
         <v>-1</v>
@@ -6442,16 +6442,16 @@
         <v>5.882697390434339</v>
       </c>
       <c r="F104" t="n">
-        <v>1.183989726946954</v>
+        <v>1.184113344748763</v>
       </c>
       <c r="G104" t="n">
-        <v>1.147418354297188</v>
+        <v>1.147543603240018</v>
       </c>
       <c r="H104" t="n">
-        <v>0.03484814820355922</v>
+        <v>0.03484780175225395</v>
       </c>
       <c r="I104" t="n">
-        <v>1.04944952702051</v>
+        <v>1.04941315290797</v>
       </c>
       <c r="J104" t="n">
         <v>-1</v>
@@ -6501,16 +6501,16 @@
         <v>5.918807384063352</v>
       </c>
       <c r="F105" t="n">
-        <v>1.177513240618361</v>
+        <v>1.177637617228203</v>
       </c>
       <c r="G105" t="n">
-        <v>1.152404569060739</v>
+        <v>1.152529747451838</v>
       </c>
       <c r="H105" t="n">
-        <v>0.03131644604906979</v>
+        <v>0.03131609126999332</v>
       </c>
       <c r="I105" t="n">
-        <v>0.8017727017388721</v>
+        <v>0.8017561821459879</v>
       </c>
       <c r="J105" t="n">
         <v>0</v>
@@ -6560,16 +6560,16 @@
         <v>5.908924968232186</v>
       </c>
       <c r="F106" t="n">
-        <v>1.12052219744635</v>
+        <v>1.120646366389124</v>
       </c>
       <c r="G106" t="n">
-        <v>1.153661534761122</v>
+        <v>1.153786632349175</v>
       </c>
       <c r="H106" t="n">
-        <v>0.0293500558619402</v>
+        <v>0.02934980069856702</v>
       </c>
       <c r="I106" t="n">
-        <v>-1.129106447723837</v>
+        <v>-1.129147904628485</v>
       </c>
       <c r="J106" t="n">
         <v>1</v>
@@ -6619,16 +6619,16 @@
         <v>5.895256457589491</v>
       </c>
       <c r="F107" t="n">
-        <v>1.147357090962278</v>
+        <v>1.14748097267776</v>
       </c>
       <c r="G107" t="n">
-        <v>1.155643324112446</v>
+        <v>1.155768319143789</v>
       </c>
       <c r="H107" t="n">
-        <v>0.02735515079521461</v>
+        <v>0.02735497342249278</v>
       </c>
       <c r="I107" t="n">
-        <v>-0.3029130861752357</v>
+        <v>-0.3029557491441568</v>
       </c>
       <c r="J107" t="n">
         <v>0</v>
@@ -6678,16 +6678,16 @@
         <v>5.897867925179888</v>
       </c>
       <c r="F108" t="n">
-        <v>1.143340433196783</v>
+        <v>1.143464369789111</v>
       </c>
       <c r="G108" t="n">
-        <v>1.155353019102058</v>
+        <v>1.155477946691243</v>
       </c>
       <c r="H108" t="n">
-        <v>0.02745834023518157</v>
+        <v>0.02745819135595296</v>
       </c>
       <c r="I108" t="n">
-        <v>-0.4374840504701717</v>
+        <v>-0.4375225136424325</v>
       </c>
       <c r="J108" t="n">
         <v>0</v>
@@ -6737,16 +6737,16 @@
         <v>5.875997591000409</v>
       </c>
       <c r="F109" t="n">
-        <v>1.120860662844942</v>
+        <v>1.120984139858534</v>
       </c>
       <c r="G109" t="n">
-        <v>1.153516085078924</v>
+        <v>1.153640925740376</v>
       </c>
       <c r="H109" t="n">
-        <v>0.02850894472430238</v>
+        <v>0.02850888661294745</v>
       </c>
       <c r="I109" t="n">
-        <v>-1.145444791092014</v>
+        <v>-1.145494958298751</v>
       </c>
       <c r="J109" t="n">
         <v>1</v>
@@ -6796,16 +6796,16 @@
         <v>5.879890291127706</v>
       </c>
       <c r="F110" t="n">
-        <v>1.140052265775034</v>
+        <v>1.140175824589031</v>
       </c>
       <c r="G110" t="n">
-        <v>1.152883031156145</v>
+        <v>1.153007748355449</v>
       </c>
       <c r="H110" t="n">
-        <v>0.02866783779096138</v>
+        <v>0.02866781056695225</v>
       </c>
       <c r="I110" t="n">
-        <v>-0.4475665543620606</v>
+        <v>-0.4476073865651421</v>
       </c>
       <c r="J110" t="n">
         <v>0</v>
@@ -6855,16 +6855,16 @@
         <v>5.885214726902118</v>
       </c>
       <c r="F111" t="n">
-        <v>1.137825816460904</v>
+        <v>1.137949487161507</v>
       </c>
       <c r="G111" t="n">
-        <v>1.149854123713858</v>
+        <v>1.149978727098074</v>
       </c>
       <c r="H111" t="n">
-        <v>0.026740598161966</v>
+        <v>0.02674047623377018</v>
       </c>
       <c r="I111" t="n">
-        <v>-0.4498144424481425</v>
+        <v>-0.4498513725561356</v>
       </c>
       <c r="J111" t="n">
         <v>0</v>
@@ -6914,16 +6914,16 @@
         <v>5.911744720499765</v>
       </c>
       <c r="F112" t="n">
-        <v>1.153725485457355</v>
+        <v>1.153849713653827</v>
       </c>
       <c r="G112" t="n">
-        <v>1.149498130758343</v>
+        <v>1.149622659501402</v>
       </c>
       <c r="H112" t="n">
-        <v>0.02663375193181083</v>
+        <v>0.02663360131760112</v>
       </c>
       <c r="I112" t="n">
-        <v>0.1587217118277306</v>
+        <v>0.1587113249169001</v>
       </c>
       <c r="J112" t="n">
         <v>0</v>
@@ -6973,16 +6973,16 @@
         <v>5.9222484364193</v>
       </c>
       <c r="F113" t="n">
-        <v>1.122245144563881</v>
+        <v>1.122369593483295</v>
       </c>
       <c r="G113" t="n">
-        <v>1.148252650829252</v>
+        <v>1.148377115543679</v>
       </c>
       <c r="H113" t="n">
-        <v>0.02732262170829436</v>
+        <v>0.02732248142851952</v>
       </c>
       <c r="I113" t="n">
-        <v>-0.9518671576628125</v>
+        <v>-0.9518726228590999</v>
       </c>
       <c r="J113" t="n">
         <v>0</v>
@@ -7020,28 +7020,28 @@
         <v>46190</v>
       </c>
       <c r="B114" t="n">
-        <v>205.3699951171875</v>
+        <v>205</v>
       </c>
       <c r="C114" t="n">
-        <v>363.614990234375</v>
+        <v>362.8299865722656</v>
       </c>
       <c r="D114" t="n">
-        <v>5.324813206576316</v>
+        <v>5.323009979138408</v>
       </c>
       <c r="E114" t="n">
-        <v>5.896095588720761</v>
+        <v>5.893934368001432</v>
       </c>
       <c r="F114" t="n">
-        <v>1.130963153834694</v>
+        <v>1.130821040961587</v>
       </c>
       <c r="G114" t="n">
-        <v>1.146987806829052</v>
+        <v>1.147098904280873</v>
       </c>
       <c r="H114" t="n">
-        <v>0.02751726673242495</v>
+        <v>0.02752534777608156</v>
       </c>
       <c r="I114" t="n">
-        <v>-0.5823490083582963</v>
+        <v>-0.5913772080812839</v>
       </c>
       <c r="J114" t="n">
         <v>0</v>
@@ -7056,10 +7056,10 @@
         <v>0</v>
       </c>
       <c r="N114" t="n">
-        <v>-0.009835632365376323</v>
+        <v>-0.01161951506464221</v>
       </c>
       <c r="O114" t="n">
-        <v>-0.02581382388647024</v>
+        <v>-0.02791698172199431</v>
       </c>
       <c r="P114" t="n">
         <v>-0</v>

</xml_diff>